<commit_message>
structure finalisation, and finalising WRF description
</commit_message>
<xml_diff>
--- a/tables/state_variables.xlsx
+++ b/tables/state_variables.xlsx
@@ -53,7 +53,7 @@
     <t xml:space="preserve">Velocities simulated by the hydrodynamic model, subject to boundary forcing</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href='hydrodynamics.html'&gt;Chapter 7&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href='hydrodynamics.html'&gt;Chapter 10&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">T</t>
@@ -107,7 +107,7 @@
     <t xml:space="preserve">Incident light attenuated as a function of depth</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href='light-climate.html'&gt;Chapter 13&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href='light-climate.html'&gt;Chapter 16&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">K_d</t>
@@ -158,7 +158,7 @@
     <t xml:space="preserve">Impacted by photosynthesis, organic decomposition, nitrification, surface exchange, and sediment oxygen demand</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href='bgc-model.html'&gt;Chapter 11&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href='bgc-model.html'&gt;Chapter 14&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">RSi</t>
@@ -359,7 +359,7 @@
     <t xml:space="preserve">Benthic photosynthesis and respiration</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href='bgc-model.html'&gt;Chapter 11&lt;/a&gt;; &lt;a href='benthic.html'&gt;Chapter 14&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href='bgc-model.html'&gt;Chapter 14&lt;/a&gt;; &lt;a href='benthic.html'&gt;Chapter 17&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">MAC_A</t>
@@ -371,7 +371,7 @@
     <t xml:space="preserve">Benthic photosynthesis, nutrient uptake, respiration</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href='benthic.html'&gt;Chapter 14&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href='benthic.html'&gt;Chapter 17&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">MAC_B</t>
@@ -401,7 +401,7 @@
     <t xml:space="preserve">Composite index based on light, temperature, substrate, wave stress, current stress</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href='habitat.html'&gt;Chapter 15&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href='habitat.html'&gt;Chapter 18&lt;/a&gt;</t>
   </si>
 </sst>
 </file>

</xml_diff>